<commit_message>
fix: republicar modelo Volcan con Kd real (8.0%→8.78%, cobertura 98.3%)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/valora-demo/modelos/volcan-modelo.xlsx
+++ b/valora-demo/modelos/volcan-modelo.xlsx
@@ -6008,11 +6008,11 @@
         </is>
       </c>
       <c r="C28" s="29" t="n">
-        <v>0.1436814077018473</v>
+        <v>0.0878</v>
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>Default: |gastos financieros| / deuda financiera promedio (histórico)</t>
+          <t>Kd real ponderado por instrumento en USD (deuda_financiera SMV, 98.3% saldo, 7/9 instrumentos (Préstamo Sindicado SOFR+500pb ex-texto nota)) — ver kd_real.py</t>
         </is>
       </c>
     </row>

</xml_diff>